<commit_message>
Peer Code Verification: two-answer chart with 1–5 rating, rename-for-sense part, four checks
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GitProject/PeerCodeVerification/assets/verification-table.xlsx
+++ b/GitProject/PeerCodeVerification/assets/verification-table.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +67,11 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -123,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,11 +148,14 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -517,15 +525,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -543,9 +548,6 @@
       </c>
       <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -559,247 +561,166 @@
         </is>
       </c>
       <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>My fork URL</t>
+          <t>My fork and branch</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/YOUR-USERNAME/git-project-THEIRNAME</t>
+          <t>https://github.com/YOUR-USERNAME/git-project-THEIRNAME/tree/peer-review-YOURNAME</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr"/>
+          <t>Rename commit URL</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/YOUR-USERNAME/git-project-THEIRNAME/commit/SHA</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="44" customHeight="1">
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>How to use this sheet: fill in the yellow cells above, then columns C–F for every numbered row. Column B is the fixed checklist — do not edit it. The grey row is an example of the level of detail expected; you may delete it. Verdict must be one of: Works · Partly · Fails · Could not test · Not implemented.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
+          <t>How to use this sheet: fill in the yellow cells above, then columns B and C for every numbered row. Column A is the fixed checklist — do not edit it. The grey row is an example of the level of detail expected; you may delete it. Rating: 5 = works exactly as described and you proved it · 4 = works, one small rule broken · 3 = partly works · 2 = runs but does the wrong thing · 1 = missing, fails, or could not be tested (say which).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="62" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Behavior to verify</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Behavior to verify</t>
+          <t>How well does it work? (1–5, 5 is best)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>How their code does it (method names, approach, data types)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>How I verified it (exact commands or calls, and what you saw)</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>What I changed to test it (or "nothing")</t>
+          <t>Is it functional / verified the functionality? What was modified to get it working?
+How their code does it (method names, approach, data types) · how you verified it (exact commands or calls, and what you saw) · what you changed to test it, or "nothing"</t>
         </is>
       </c>
     </row>
     <row r="9" ht="118" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Ex.</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
           <t>Example (not graded): Hashing an empty file — the blob for a 0-byte file is named da39a3ee5e6b4b0d3255bfef95601890afd80709.</t>
         </is>
       </c>
+      <c r="B9" s="9" t="n">
+        <v>5</v>
+      </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Works</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>hashFile(File f) reads all bytes with Files.readAllBytes, feeds them to MessageDigest.getInstance("SHA-1"), and converts the byte[] to hex with String.format("%02x", b) in a loop. add(String path) calls hashFile, then writeBlob, then updateIndex.</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>printf '' &gt; empty.txt ; wc -c empty.txt → 0 ; shasum empty.txt → da39a3ee5e6b4b0d3255bfef95601890afd80709. Ran Verify.java (init, then add("empty.txt")). ls git/objects → da39a3ee5e6b4b0d3255bfef95601890afd80709 ; cat -e git/index → da39a3ee...0709 empty.txt$</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Added Verify.java with a main() that calls init() and add("empty.txt"). Did not edit Git.java.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="130" customHeight="1">
-      <c r="A10" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Initialize — init() creates git/, git/objects/, git/index, and git/HEAD. Running it a second time reports that the repository already exists and changes nothing.</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-    </row>
-    <row r="11" ht="130" customHeight="1">
-      <c r="A11" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Stage a file into a blob — Adding a file creates git/objects/&lt;hash&gt; whose content is byte for byte identical to the original file.</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-    </row>
-    <row r="12" ht="130" customHeight="1">
-      <c r="A12" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Hash correctness — The blob's filename is the true SHA-1 of the content. A file containing exactly sha1test (8 bytes, no newline) must produce 12c4c60ee087ae0f12dc6abc88495e459f6f2654 — the same as   printf 'sha1test' | shasum   or   echo -n "sha1test" | sha1sum</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-    </row>
-    <row r="13" ht="130" customHeight="1">
-      <c r="A13" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Index tracks the file — After adding a file, git/index contains a line for that file.</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-    </row>
-    <row r="14" ht="130" customHeight="1">
-      <c r="A14" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Index line format — Each line is &lt;hash&gt;, one space, &lt;relative path&gt;. The hash matches the blob's filename. No trailing space. No blank final line.</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-    </row>
-    <row r="15" ht="130" customHeight="1">
-      <c r="A15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Multiple entries — Adding several different files produces one correct line per file, each on its own line.</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-    </row>
-    <row r="16" ht="130" customHeight="1">
-      <c r="A16" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Duplicate content — Two files with identical content at different paths produce two index lines with the same hash but exactly one blob in git/objects/.</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-    </row>
-    <row r="17" ht="130" customHeight="1">
-      <c r="A17" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Modify and re-add — Changing a file's content and adding it again replaces its index line with the new hash (no duplicate path) and writes a new blob. The old blob remains.</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-    </row>
-    <row r="18" ht="130" customHeight="1">
-      <c r="A18" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Compression — Blob content is compressed on disk and decompresses back to the original. (Optional stretch milestone — 'Not implemented' is a legitimate verdict.)</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
+          <t>Functional, verified. hashFile(File f) reads all bytes with Files.readAllBytes, feeds them to MessageDigest.getInstance("SHA-1"), and converts the byte[] to hex with String.format("%02x", b) in a loop; add(String path) calls hashFile, then writeBlob, then updateIndex. Verified: printf '' &gt; empty.txt ; wc -c empty.txt → 0 ; shasum empty.txt → da39a3ee...0709. Ran Verify.java (init, then add("empty.txt")). ls git/objects → da39a3ee5e6b4b0d3255bfef95601890afd80709 ; cat -e git/index → da39a3ee...0709 empty.txt$ . Modified: added Verify.java with a main() that calls init() and add("empty.txt"). Did not edit Git.java.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>1. Initialize — init() creates git/, git/objects/, git/index, and git/HEAD. Running it a second time reports that the repository already exists and changes nothing.</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="12" t="n"/>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>2. Stage a file into a blob — Adding a file creates git/objects/&lt;hash&gt; whose content is byte for byte identical to the original file.</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="12" t="n"/>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>3. Hash correctness — The blob's filename is the true SHA-1 of the content. A file containing exactly sha1test (8 bytes, no newline) must produce 12c4c60ee087ae0f12dc6abc88495e459f6f2654 — the same as   printf 'sha1test' | shasum   or   echo -n "sha1test" | sha1sum</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>4. Index tracks the file — After adding a file, git/index contains a line for that file.</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="12" t="n"/>
+    </row>
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>5. Index line format — Each line is &lt;hash&gt;, one space, &lt;relative path&gt;. The hash matches the blob's filename. No trailing space. No blank final line.</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="12" t="n"/>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>6. Multiple entries — Adding several different files produces one correct line per file, each on its own line.</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="12" t="n"/>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>7. Duplicate content — Two files with identical content at different paths produce two index lines with the same hash but exactly one blob in git/objects/.</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="12" t="n"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>8. Modify and re-add — Changing a file's content and adding it again replaces its index line with the new hash (no duplicate path) and writes a new blob. The old blob remains.</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>9. Compression — Blob content is compressed on disk and decompresses back to the original. (Optional stretch milestone — a 1 with the note 'not implemented' is a complete answer.)</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C10:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Verdict" error="Choose one of: Works, Partly, Fails, Could not test, Not implemented" type="list">
-      <formula1>"Works,Partly,Fails,Could not test,Not implemented"</formula1>
+    <dataValidation sqref="B10:B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rating" error="Enter a whole number from 1 (worst) to 5 (best)" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update assignment for Topics Quiz for Git Project phase 1
</commit_message>
<xml_diff>
--- a/GitProject/PeerCodeVerification/assets/verification-table.xlsx
+++ b/GitProject/PeerCodeVerification/assets/verification-table.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -667,7 +667,7 @@
     <row r="14" ht="150" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>5. Index line format — Each line is &lt;hash&gt;, one space, &lt;relative path&gt;. The hash matches the blob's filename. No trailing space. No blank final line.</t>
+          <t>5. Duplicate content — Two files with identical content at different paths produce two index lines with the same hash but exactly one blob in git/objects/.</t>
         </is>
       </c>
       <c r="B14" s="11" t="n"/>
@@ -676,38 +676,11 @@
     <row r="15" ht="150" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>6. Multiple entries — Adding several different files produces one correct line per file, each on its own line.</t>
+          <t>6. Compression — Blob content is compressed on disk and decompresses back to the original. (Optional stretch milestone — a 1 with the note 'not implemented' is a complete answer.)</t>
         </is>
       </c>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="12" t="n"/>
-    </row>
-    <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>7. Duplicate content — Two files with identical content at different paths produce two index lines with the same hash but exactly one blob in git/objects/.</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="12" t="n"/>
-    </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>8. Modify and re-add — Changing a file's content and adding it again replaces its index line with the new hash (no duplicate path) and writes a new blob. The old blob remains.</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="12" t="n"/>
-    </row>
-    <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>9. Compression — Blob content is compressed on disk and decompresses back to the original. (Optional stretch milestone — a 1 with the note 'not implemented' is a complete answer.)</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -719,7 +692,7 @@
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B10:B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rating" error="Enter a whole number from 1 (worst) to 5 (best)" type="list">
+    <dataValidation sqref="B10:B15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Rating" error="Enter a whole number from 1 (worst) to 5 (best)" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update peer review for git
</commit_message>
<xml_diff>
--- a/GitProject/PeerCodeVerification/assets/verification-table.xlsx
+++ b/GitProject/PeerCodeVerification/assets/verification-table.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/THEIR-USERNAME/git-project-THEIRNAME</t>
+          <t>https://github.com/THEIR-USERNAME/THEIR-REPO-NAME</t>
         </is>
       </c>
       <c r="C3" s="4" t="n"/>
@@ -570,7 +570,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/YOUR-USERNAME/git-project-THEIRNAME/tree/peer-review-YOURNAME</t>
+          <t>https://github.com/YOUR-USERNAME/THEIR-REPO-NAME/tree/peer-review-YOURNAME</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -583,7 +583,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/YOUR-USERNAME/git-project-THEIRNAME/commit/SHA</t>
+          <t>https://github.com/YOUR-USERNAME/THEIR-REPO-NAME/commit/SHA</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>

</xml_diff>